<commit_message>
queue examples 저장, csv 버전과 xlsx 버전 모두 저장
</commit_message>
<xml_diff>
--- a/script/simulation_queue_example_xlsx.xlsx
+++ b/script/simulation_queue_example_xlsx.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f03addda2663411/SRBL/WearableOptimizedControl/Optimizer/Moco_git/script/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="8_{985CFB64-8444-49E3-9649-B21738068EB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBBE317C-02E5-419D-8550-0F02E387FD3B}"/>
+  <xr:revisionPtr revIDLastSave="84" documentId="8_{985CFB64-8444-49E3-9649-B21738068EB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C1BAE2F-5D5A-46BB-8E3D-22D3FA48E861}"/>
   <bookViews>
-    <workbookView xWindow="285" yWindow="1830" windowWidth="26595" windowHeight="13770" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="simulation_queue" sheetId="1" r:id="rId1"/>
-    <sheet name="Completed_queue" sheetId="2" r:id="rId2"/>
+    <sheet name="completed_queue" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="59">
   <si>
     <t>SF</t>
   </si>
@@ -142,30 +142,6 @@
     <t>modeAsym</t>
   </si>
   <si>
-    <t>default QP_effort = 0.01</t>
-  </si>
-  <si>
-    <t>default QP_smooth = 0</t>
-  </si>
-  <si>
-    <t>default mocoEffort = 1</t>
-  </si>
-  <si>
-    <t>default mocoFinalTime = 0.03</t>
-  </si>
-  <si>
-    <t>default mocoTimeBound = [0.4 0.8]</t>
-  </si>
-  <si>
-    <t>default mocoDistBound = [0.4 1.0]</t>
-  </si>
-  <si>
-    <t>default gaitMode = modeSym</t>
-  </si>
-  <si>
-    <t>ID rule : 'S(Sym)/A(Asym)' + 'F(Off)/W(WoC)/P(Spline)' + 'index number' + '-iter number' (e.g. modeSym + modeWoC + 1st tiral + 5 iter = SW001-5)</t>
-  </si>
-  <si>
     <t>SW001-1</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -178,27 +154,84 @@
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
-    <t>test1</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
-    <t>test2</t>
-  </si>
-  <si>
-    <t>test3</t>
-  </si>
-  <si>
-    <t>test4</t>
-  </si>
-  <si>
-    <t>test5</t>
-  </si>
-  <si>
     <t>SW002-1</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
   <si>
     <t>AW001-1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>test1-2</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>test2-2</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>test3-2</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>test4-2</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>test5-2</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>ID rule : 
+'S(Sym)/A(Asym)' 
++ 'F(Off)/W(WoC)/P(Spline)' 
++ 'index number' 
++ '-iter number' 
+(e.g. modeSym 
++ modeWoC 
++ 1st tiral 
++ 5 iter 
+= SW001-5)</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">default QP_effort </t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>[0.4 0.8]</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>[0.4 1.0]</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>modeSym'</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>default QP_smooth</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>default mocoEffort</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>default mocoFinalTime</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>default mocoTimeBound</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>default mocoDistBound</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>default gaitMode</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -416,13 +449,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
+        <fgColor theme="4" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
+        <fgColor theme="4" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -439,13 +472,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
+        <fgColor theme="5" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
+        <fgColor theme="5" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -462,13 +495,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
+        <fgColor theme="6" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
+        <fgColor theme="6" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -485,13 +518,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor theme="7" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
+        <fgColor theme="7" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -508,13 +541,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
+        <fgColor theme="8" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
+        <fgColor theme="8" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -531,13 +564,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
+        <fgColor theme="9" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
+        <fgColor theme="9" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -570,7 +603,7 @@
       <right/>
       <top/>
       <bottom style="thick">
-        <color theme="4" tint="0.499984740745262"/>
+        <color theme="4" tint="0.49995422223578601"/>
       </bottom>
       <diagonal/>
     </border>
@@ -792,8 +825,17 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1151,59 +1193,105 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U15"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="27.375" customWidth="1"/>
+    <col min="2" max="2" width="13.125" customWidth="1"/>
+    <col min="3" max="3" width="22.375" customWidth="1"/>
+    <col min="4" max="4" width="8.25" customWidth="1"/>
+    <col min="5" max="5" width="13.5" customWidth="1"/>
+    <col min="6" max="6" width="6.875" customWidth="1"/>
+    <col min="7" max="7" width="4.125" customWidth="1"/>
+    <col min="8" max="8" width="4" customWidth="1"/>
+    <col min="9" max="9" width="3.875" customWidth="1"/>
+    <col min="10" max="10" width="7.5" customWidth="1"/>
+    <col min="11" max="11" width="11.375" customWidth="1"/>
+    <col min="12" max="12" width="9.25" customWidth="1"/>
+    <col min="13" max="13" width="11" customWidth="1"/>
+    <col min="14" max="14" width="4.625" customWidth="1"/>
+    <col min="15" max="15" width="10.625" customWidth="1"/>
+    <col min="16" max="16" width="14.125" customWidth="1"/>
+    <col min="17" max="17" width="15.75" customWidth="1"/>
+    <col min="18" max="18" width="14.875" customWidth="1"/>
+    <col min="19" max="19" width="9.5" customWidth="1"/>
+    <col min="20" max="20" width="12.875" customWidth="1"/>
+    <col min="21" max="21" width="9.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>38</v>
+      <c r="A1" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="2">
+        <v>0.01</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>39</v>
+      <c r="A2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="2">
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>40</v>
+      <c r="A3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="2">
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>41</v>
+      <c r="A4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0.03</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>42</v>
+      <c r="A5" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>43</v>
+      <c r="A6" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>45</v>
-      </c>
+      <c r="A7" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" ht="165" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="2"/>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="A9" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="B9" s="2"/>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C10" t="s">
@@ -1265,11 +1353,11 @@
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>46</v>
-      </c>
-      <c r="B11">
-        <v>260415</v>
+      <c r="A11" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="2">
+        <v>260416</v>
       </c>
       <c r="C11" t="s">
         <v>28</v>
@@ -1281,7 +1369,7 @@
         <v>29</v>
       </c>
       <c r="K11" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="L11">
         <v>0.01</v>
@@ -1293,140 +1381,6 @@
         <v>31</v>
       </c>
       <c r="U11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>47</v>
-      </c>
-      <c r="B12">
-        <v>260415</v>
-      </c>
-      <c r="C12" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12">
-        <v>1</v>
-      </c>
-      <c r="E12" t="s">
-        <v>33</v>
-      </c>
-      <c r="K12" t="s">
-        <v>50</v>
-      </c>
-      <c r="S12" t="s">
-        <v>31</v>
-      </c>
-      <c r="U12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>48</v>
-      </c>
-      <c r="B13">
-        <v>260415</v>
-      </c>
-      <c r="C13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D13">
-        <v>1</v>
-      </c>
-      <c r="E13" t="s">
-        <v>35</v>
-      </c>
-      <c r="F13">
-        <v>0.1</v>
-      </c>
-      <c r="G13">
-        <v>0.1</v>
-      </c>
-      <c r="H13">
-        <v>0.2</v>
-      </c>
-      <c r="I13">
-        <v>0.1</v>
-      </c>
-      <c r="J13">
-        <v>0.8</v>
-      </c>
-      <c r="K13" t="s">
-        <v>51</v>
-      </c>
-      <c r="S13" t="s">
-        <v>31</v>
-      </c>
-      <c r="U13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14">
-        <v>260415</v>
-      </c>
-      <c r="C14" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14">
-        <v>1</v>
-      </c>
-      <c r="E14" t="s">
-        <v>29</v>
-      </c>
-      <c r="K14" t="s">
-        <v>52</v>
-      </c>
-      <c r="L14">
-        <v>0.01</v>
-      </c>
-      <c r="M14">
-        <v>0</v>
-      </c>
-      <c r="S14" t="s">
-        <v>31</v>
-      </c>
-      <c r="T14" t="s">
-        <v>36</v>
-      </c>
-      <c r="U14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>55</v>
-      </c>
-      <c r="B15">
-        <v>260415</v>
-      </c>
-      <c r="C15" t="s">
-        <v>28</v>
-      </c>
-      <c r="D15">
-        <v>1</v>
-      </c>
-      <c r="E15" t="s">
-        <v>29</v>
-      </c>
-      <c r="K15" t="s">
-        <v>53</v>
-      </c>
-      <c r="L15">
-        <v>0.01</v>
-      </c>
-      <c r="M15">
-        <v>0</v>
-      </c>
-      <c r="S15" t="s">
-        <v>37</v>
-      </c>
-      <c r="U15">
         <v>0</v>
       </c>
     </row>
@@ -1439,15 +1393,38 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFFA8AF3-BD89-432D-8740-30DBF5179C15}">
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U14"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.375" customWidth="1"/>
+    <col min="2" max="2" width="7.25" customWidth="1"/>
+    <col min="3" max="3" width="24.75" customWidth="1"/>
+    <col min="4" max="4" width="4" customWidth="1"/>
+    <col min="5" max="5" width="13.5" customWidth="1"/>
+    <col min="6" max="6" width="6.875" customWidth="1"/>
+    <col min="7" max="7" width="4.125" customWidth="1"/>
+    <col min="8" max="8" width="4" customWidth="1"/>
+    <col min="9" max="9" width="3.875" customWidth="1"/>
+    <col min="10" max="10" width="7.5" customWidth="1"/>
+    <col min="11" max="11" width="14.25" customWidth="1"/>
+    <col min="12" max="12" width="9.25" customWidth="1"/>
+    <col min="13" max="13" width="11" customWidth="1"/>
+    <col min="14" max="14" width="4.625" customWidth="1"/>
+    <col min="15" max="15" width="10.625" customWidth="1"/>
+    <col min="16" max="16" width="14.125" customWidth="1"/>
+    <col min="17" max="17" width="15.75" customWidth="1"/>
+    <col min="18" max="18" width="14.875" customWidth="1"/>
+    <col min="19" max="19" width="9.625" customWidth="1"/>
+    <col min="20" max="20" width="12.875" customWidth="1"/>
+    <col min="21" max="21" width="9.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.3">
@@ -1455,7 +1432,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.3">
@@ -1463,7 +1440,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.3">
@@ -1479,7 +1456,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
@@ -1562,7 +1539,7 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B9">
         <v>260415</v>
@@ -1589,6 +1566,172 @@
         <v>31</v>
       </c>
       <c r="U9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10">
+        <v>260415</v>
+      </c>
+      <c r="C10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>29</v>
+      </c>
+      <c r="K10" t="s">
+        <v>43</v>
+      </c>
+      <c r="L10">
+        <v>0.01</v>
+      </c>
+      <c r="M10">
+        <v>1</v>
+      </c>
+      <c r="S10" t="s">
+        <v>31</v>
+      </c>
+      <c r="U10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11">
+        <v>260415</v>
+      </c>
+      <c r="C11" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11" t="s">
+        <v>33</v>
+      </c>
+      <c r="K11" t="s">
+        <v>44</v>
+      </c>
+      <c r="S11" t="s">
+        <v>31</v>
+      </c>
+      <c r="U11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12">
+        <v>260415</v>
+      </c>
+      <c r="C12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12">
+        <v>0.1</v>
+      </c>
+      <c r="G12">
+        <v>0.1</v>
+      </c>
+      <c r="H12">
+        <v>0.2</v>
+      </c>
+      <c r="I12">
+        <v>0.1</v>
+      </c>
+      <c r="J12">
+        <v>0.8</v>
+      </c>
+      <c r="K12" t="s">
+        <v>45</v>
+      </c>
+      <c r="S12" t="s">
+        <v>31</v>
+      </c>
+      <c r="U12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13">
+        <v>260415</v>
+      </c>
+      <c r="C13" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13" t="s">
+        <v>29</v>
+      </c>
+      <c r="K13" t="s">
+        <v>46</v>
+      </c>
+      <c r="L13">
+        <v>0.01</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="S13" t="s">
+        <v>31</v>
+      </c>
+      <c r="T13" t="s">
+        <v>36</v>
+      </c>
+      <c r="U13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14">
+        <v>260415</v>
+      </c>
+      <c r="C14" t="s">
+        <v>28</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" t="s">
+        <v>29</v>
+      </c>
+      <c r="K14" t="s">
+        <v>47</v>
+      </c>
+      <c r="L14">
+        <v>0.01</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="S14" t="s">
+        <v>37</v>
+      </c>
+      <c r="U14">
         <v>1</v>
       </c>
     </row>

</xml_diff>